<commit_message>
Refactor main.py：微調 calc_late、calc_early 與 _get_shift_rules
- 修改 `calc_late`，大於 0 才回傳 `late_min`，否則回傳 '-'
- 修改 `calc_early`，依 shift code 計算提早下班分鐘
- 調整 `_get_shift_rules`，A1 & A2 班別上班時間改為 7:50 AM
</commit_message>
<xml_diff>
--- a/output/Master_Report.xlsx
+++ b/output/Master_Report.xlsx
@@ -732,7 +732,7 @@
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
@@ -741,10 +741,10 @@
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>141</v>
+        <v>67</v>
       </c>
       <c r="T2" t="n">
-        <v>34</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3">
@@ -792,7 +792,7 @@
         <v>1</v>
       </c>
       <c r="O3" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
@@ -801,10 +801,10 @@
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>621</v>
+        <v>571</v>
       </c>
       <c r="T3" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4">
@@ -834,7 +834,7 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" s="10" t="n"/>
       <c r="H4" t="n">
-        <v>16.5</v>
+        <v>16</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -846,13 +846,13 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>16.5</v>
+        <v>16</v>
       </c>
       <c r="N4" t="n">
         <v>3</v>
       </c>
       <c r="O4" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
@@ -861,10 +861,10 @@
         <v>2</v>
       </c>
       <c r="S4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>0</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5">
@@ -894,7 +894,7 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" s="10" t="n"/>
       <c r="H5" t="n">
-        <v>27.5</v>
+        <v>27</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -906,7 +906,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>27.5</v>
+        <v>27</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -924,7 +924,7 @@
         <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6">
@@ -954,7 +954,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" s="10" t="n"/>
       <c r="H6" t="n">
-        <v>14.5</v>
+        <v>14</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -966,7 +966,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>14.5</v>
+        <v>14</v>
       </c>
       <c r="N6" t="n">
         <v>3</v>
@@ -981,10 +981,10 @@
         <v>2</v>
       </c>
       <c r="S6" t="n">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="T6" t="n">
-        <v>318</v>
+        <v>434</v>
       </c>
     </row>
     <row r="7">
@@ -1041,10 +1041,10 @@
         <v>2</v>
       </c>
       <c r="S7" t="n">
-        <v>5051</v>
+        <v>4981</v>
       </c>
       <c r="T7" t="n">
-        <v>3709</v>
+        <v>3949</v>
       </c>
     </row>
     <row r="8">
@@ -1092,7 +1092,7 @@
         <v>2</v>
       </c>
       <c r="O8" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="P8" t="n">
         <v>0</v>
@@ -1101,10 +1101,10 @@
         <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>67</v>
+        <v>14</v>
       </c>
       <c r="T8" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9">
@@ -1214,7 +1214,7 @@
         <v>1</v>
       </c>
       <c r="O10" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1223,10 +1223,10 @@
         <v>1</v>
       </c>
       <c r="S10" t="n">
-        <v>157</v>
+        <v>67</v>
       </c>
       <c r="T10" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11">
@@ -1256,7 +1256,7 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" s="10" t="n"/>
       <c r="H11" t="n">
-        <v>27</v>
+        <v>26.5</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -1268,13 +1268,13 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>27</v>
+        <v>26.5</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
@@ -1283,10 +1283,10 @@
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>85</v>
+        <v>23</v>
       </c>
       <c r="T11" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12">
@@ -1334,7 +1334,7 @@
         <v>2</v>
       </c>
       <c r="O12" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
@@ -1343,10 +1343,10 @@
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>669</v>
+        <v>606</v>
       </c>
       <c r="T12" t="n">
-        <v>0</v>
+        <v>93</v>
       </c>
     </row>
     <row r="13">
@@ -1376,7 +1376,7 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" s="10" t="n"/>
       <c r="H13" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -1388,13 +1388,13 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
@@ -1403,10 +1403,10 @@
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14">
@@ -1454,7 +1454,7 @@
         <v>2</v>
       </c>
       <c r="O14" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
@@ -1463,10 +1463,10 @@
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15">
@@ -1523,10 +1523,10 @@
         <v>1</v>
       </c>
       <c r="S15" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="T15" t="n">
-        <v>319</v>
+        <v>398</v>
       </c>
     </row>
     <row r="16">
@@ -1556,7 +1556,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" s="10" t="n"/>
       <c r="H16" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -1568,7 +1568,7 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="N16" t="n">
         <v>2</v>
@@ -1583,10 +1583,10 @@
         <v>1</v>
       </c>
       <c r="S16" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="T16" t="n">
-        <v>657</v>
+        <v>775</v>
       </c>
     </row>
     <row r="17">
@@ -1646,7 +1646,7 @@
         <v>0</v>
       </c>
       <c r="T17" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18">
@@ -1676,7 +1676,7 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" s="10" t="n"/>
       <c r="H18" t="n">
-        <v>25.5</v>
+        <v>25</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
@@ -1688,13 +1688,13 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>25.5</v>
+        <v>25</v>
       </c>
       <c r="N18" t="n">
         <v>2</v>
       </c>
       <c r="O18" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1703,10 +1703,10 @@
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>65</v>
+        <v>2</v>
       </c>
       <c r="T18" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
     </row>
     <row r="19">
@@ -1754,7 +1754,7 @@
         <v>1</v>
       </c>
       <c r="O19" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
@@ -1763,10 +1763,10 @@
         <v>1</v>
       </c>
       <c r="S19" t="n">
-        <v>879</v>
+        <v>843</v>
       </c>
       <c r="T19" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20">
@@ -1814,7 +1814,7 @@
         <v>1</v>
       </c>
       <c r="O20" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
@@ -1823,10 +1823,10 @@
         <v>1</v>
       </c>
       <c r="S20" t="n">
-        <v>118</v>
+        <v>10</v>
       </c>
       <c r="T20" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
     </row>
     <row r="21">
@@ -1856,7 +1856,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" s="10" t="n"/>
       <c r="H21" t="n">
-        <v>19</v>
+        <v>18.5</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -1868,13 +1868,13 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>19</v>
+        <v>18.5</v>
       </c>
       <c r="N21" t="n">
         <v>2</v>
       </c>
       <c r="O21" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="P21" t="n">
         <v>0</v>
@@ -1883,10 +1883,10 @@
         <v>2</v>
       </c>
       <c r="S21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T21" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22">
@@ -1934,7 +1934,7 @@
         <v>4</v>
       </c>
       <c r="O22" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="P22" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
         <v>2</v>
       </c>
       <c r="S22" t="n">
-        <v>134</v>
+        <v>105</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -1976,7 +1976,7 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" s="10" t="n"/>
       <c r="H23" t="n">
-        <v>15.5</v>
+        <v>15</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -1988,13 +1988,13 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>15.5</v>
+        <v>15</v>
       </c>
       <c r="N23" t="n">
         <v>1</v>
       </c>
       <c r="O23" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="P23" t="n">
         <v>0</v>
@@ -2003,10 +2003,10 @@
         <v>2</v>
       </c>
       <c r="S23" t="n">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="T23" t="n">
-        <v>0</v>
+        <v>103</v>
       </c>
     </row>
     <row r="24">
@@ -2054,7 +2054,7 @@
         <v>2</v>
       </c>
       <c r="O24" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="P24" t="n">
         <v>0</v>
@@ -2063,10 +2063,10 @@
         <v>2</v>
       </c>
       <c r="S24" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="T24" t="n">
-        <v>0</v>
+        <v>154</v>
       </c>
     </row>
     <row r="25">
@@ -2096,7 +2096,7 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" s="10" t="n"/>
       <c r="H25" t="n">
-        <v>17.5</v>
+        <v>17</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -2108,13 +2108,13 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>17.5</v>
+        <v>17</v>
       </c>
       <c r="N25" t="n">
         <v>1</v>
       </c>
       <c r="O25" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="P25" t="n">
         <v>0</v>
@@ -2123,10 +2123,10 @@
         <v>2</v>
       </c>
       <c r="S25" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="T25" t="n">
-        <v>309</v>
+        <v>424</v>
       </c>
     </row>
     <row r="26">
@@ -2174,7 +2174,7 @@
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2183,10 +2183,10 @@
         <v>1</v>
       </c>
       <c r="S26" t="n">
+        <v>13</v>
+      </c>
+      <c r="T26" t="n">
         <v>39</v>
-      </c>
-      <c r="T26" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -2234,7 +2234,7 @@
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2243,10 +2243,10 @@
         <v>1</v>
       </c>
       <c r="S27" t="n">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="T27" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="28">
@@ -2294,7 +2294,7 @@
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2303,10 +2303,10 @@
         <v>1</v>
       </c>
       <c r="S28" t="n">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="T28" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="29">
@@ -2354,7 +2354,7 @@
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2363,10 +2363,10 @@
         <v>1</v>
       </c>
       <c r="S29" t="n">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="T29" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="30">
@@ -2414,7 +2414,7 @@
         <v>0</v>
       </c>
       <c r="O30" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="P30" t="n">
         <v>0</v>
@@ -2423,10 +2423,10 @@
         <v>1</v>
       </c>
       <c r="S30" t="n">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="T30" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="31">
@@ -2474,7 +2474,7 @@
         <v>1</v>
       </c>
       <c r="O31" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="P31" t="n">
         <v>0</v>
@@ -2483,10 +2483,10 @@
         <v>1</v>
       </c>
       <c r="S31" t="n">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="T31" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32">
@@ -2534,7 +2534,7 @@
         <v>0</v>
       </c>
       <c r="O32" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="P32" t="n">
         <v>0</v>
@@ -2543,10 +2543,10 @@
         <v>1</v>
       </c>
       <c r="S32" t="n">
-        <v>757</v>
+        <v>716</v>
       </c>
       <c r="T32" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="33">
@@ -2594,7 +2594,7 @@
         <v>0</v>
       </c>
       <c r="O33" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="P33" t="n">
         <v>0</v>
@@ -2603,10 +2603,10 @@
         <v>1</v>
       </c>
       <c r="S33" t="n">
-        <v>759</v>
+        <v>718</v>
       </c>
       <c r="T33" t="n">
-        <v>618</v>
+        <v>697</v>
       </c>
     </row>
     <row r="34">
@@ -2654,7 +2654,7 @@
         <v>1</v>
       </c>
       <c r="O34" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="P34" t="n">
         <v>0</v>
@@ -2663,10 +2663,10 @@
         <v>1</v>
       </c>
       <c r="S34" t="n">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="T34" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="35">
@@ -2714,7 +2714,7 @@
         <v>0</v>
       </c>
       <c r="O35" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="P35" t="n">
         <v>0</v>
@@ -2723,10 +2723,10 @@
         <v>1</v>
       </c>
       <c r="S35" t="n">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="T35" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="36">
@@ -2774,7 +2774,7 @@
         <v>1</v>
       </c>
       <c r="O36" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="P36" t="n">
         <v>0</v>
@@ -2783,10 +2783,10 @@
         <v>1</v>
       </c>
       <c r="S36" t="n">
-        <v>354</v>
+        <v>283</v>
       </c>
       <c r="T36" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
     </row>
     <row r="37">
@@ -2878,7 +2878,7 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" s="10" t="n"/>
       <c r="H38" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
@@ -2890,13 +2890,13 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="N38" t="n">
         <v>1</v>
       </c>
       <c r="O38" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="P38" t="n">
         <v>0</v>
@@ -2905,10 +2905,10 @@
         <v>1</v>
       </c>
       <c r="S38" t="n">
-        <v>663</v>
+        <v>581</v>
       </c>
       <c r="T38" t="n">
-        <v>613</v>
+        <v>720</v>
       </c>
     </row>
     <row r="39">
@@ -2938,7 +2938,7 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" s="10" t="n"/>
       <c r="H39" t="n">
-        <v>12.5</v>
+        <v>12</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
@@ -2950,13 +2950,13 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>12.5</v>
+        <v>12</v>
       </c>
       <c r="N39" t="n">
         <v>2</v>
       </c>
       <c r="O39" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="P39" t="n">
         <v>0</v>
@@ -2965,10 +2965,10 @@
         <v>2</v>
       </c>
       <c r="S39" t="n">
-        <v>166</v>
+        <v>140</v>
       </c>
       <c r="T39" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
     </row>
     <row r="40">
@@ -3016,7 +3016,7 @@
         <v>0</v>
       </c>
       <c r="O40" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="P40" t="n">
         <v>0</v>
@@ -3025,10 +3025,10 @@
         <v>1</v>
       </c>
       <c r="S40" t="n">
-        <v>945</v>
+        <v>860</v>
       </c>
       <c r="T40" t="n">
-        <v>927</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="41">
@@ -3076,7 +3076,7 @@
         <v>2</v>
       </c>
       <c r="O41" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="P41" t="n">
         <v>0</v>
@@ -3085,10 +3085,10 @@
         <v>2</v>
       </c>
       <c r="S41" t="n">
-        <v>131</v>
+        <v>40</v>
       </c>
       <c r="T41" t="n">
-        <v>0</v>
+        <v>142</v>
       </c>
     </row>
     <row r="42">
@@ -3118,7 +3118,7 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" s="10" t="n"/>
       <c r="H42" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I42" t="n">
         <v>0</v>
@@ -3130,7 +3130,7 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="N42" t="n">
         <v>2</v>
@@ -3145,10 +3145,10 @@
         <v>1</v>
       </c>
       <c r="S42" t="n">
-        <v>471</v>
+        <v>461</v>
       </c>
       <c r="T42" t="n">
-        <v>179</v>
+        <v>372</v>
       </c>
     </row>
     <row r="43">
@@ -3207,7 +3207,7 @@
         <v>1</v>
       </c>
       <c r="S43" t="n">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="T43" t="n">
         <v>0</v>
@@ -3258,7 +3258,7 @@
         <v>2</v>
       </c>
       <c r="O44" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="P44" t="n">
         <v>0</v>
@@ -3267,10 +3267,10 @@
         <v>1</v>
       </c>
       <c r="S44" t="n">
-        <v>173</v>
+        <v>155</v>
       </c>
       <c r="T44" t="n">
-        <v>337</v>
+        <v>446</v>
       </c>
     </row>
     <row r="45">
@@ -3330,7 +3330,7 @@
         <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
     </row>
     <row r="46">
@@ -3390,7 +3390,7 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="47">
@@ -3450,7 +3450,7 @@
         <v>0</v>
       </c>
       <c r="T47" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="48">
@@ -3498,7 +3498,7 @@
         <v>2</v>
       </c>
       <c r="O48" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="P48" t="n">
         <v>0</v>
@@ -3507,10 +3507,10 @@
         <v>1</v>
       </c>
       <c r="S48" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="T48" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
     </row>
     <row r="49">
@@ -3558,7 +3558,7 @@
         <v>3</v>
       </c>
       <c r="O49" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="P49" t="n">
         <v>0</v>
@@ -3567,10 +3567,10 @@
         <v>3</v>
       </c>
       <c r="S49" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="T49" t="n">
-        <v>147</v>
+        <v>222</v>
       </c>
     </row>
     <row r="50">
@@ -3600,7 +3600,7 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" s="10" t="n"/>
       <c r="H50" t="n">
-        <v>17.5</v>
+        <v>17</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>
@@ -3612,13 +3612,13 @@
         <v>0</v>
       </c>
       <c r="L50" t="n">
-        <v>17.5</v>
+        <v>17</v>
       </c>
       <c r="N50" t="n">
         <v>1</v>
       </c>
       <c r="O50" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="P50" t="n">
         <v>0</v>
@@ -3627,10 +3627,10 @@
         <v>2</v>
       </c>
       <c r="S50" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="T50" t="n">
-        <v>0</v>
+        <v>111</v>
       </c>
     </row>
     <row r="51">
@@ -3660,7 +3660,7 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" s="10" t="n"/>
       <c r="H51" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I51" t="n">
         <v>0</v>
@@ -3672,7 +3672,7 @@
         <v>0</v>
       </c>
       <c r="L51" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="N51" t="n">
         <v>0</v>
@@ -3687,10 +3687,10 @@
         <v>2</v>
       </c>
       <c r="S51" t="n">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="T51" t="n">
-        <v>147</v>
+        <v>258</v>
       </c>
     </row>
     <row r="52">
@@ -3738,7 +3738,7 @@
         <v>0</v>
       </c>
       <c r="O52" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="P52" t="n">
         <v>0</v>
@@ -3747,10 +3747,10 @@
         <v>2</v>
       </c>
       <c r="S52" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="53">
@@ -3780,7 +3780,7 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" s="10" t="n"/>
       <c r="H53" t="n">
-        <v>32.5</v>
+        <v>32</v>
       </c>
       <c r="I53" t="n">
         <v>0</v>
@@ -3792,7 +3792,7 @@
         <v>0</v>
       </c>
       <c r="L53" t="n">
-        <v>32.5</v>
+        <v>32</v>
       </c>
       <c r="N53" t="n">
         <v>1</v>
@@ -3810,7 +3810,7 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>741</v>
+        <v>856</v>
       </c>
     </row>
     <row r="54">
@@ -3840,7 +3840,7 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" s="10" t="n"/>
       <c r="H54" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="I54" t="n">
         <v>0</v>
@@ -3852,13 +3852,13 @@
         <v>0</v>
       </c>
       <c r="L54" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="N54" t="n">
         <v>0</v>
       </c>
       <c r="O54" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="P54" t="n">
         <v>0</v>
@@ -3867,10 +3867,10 @@
         <v>1</v>
       </c>
       <c r="S54" t="n">
-        <v>457</v>
+        <v>425</v>
       </c>
       <c r="T54" t="n">
-        <v>610</v>
+        <v>689</v>
       </c>
     </row>
     <row r="55">
@@ -3918,7 +3918,7 @@
         <v>2</v>
       </c>
       <c r="O55" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="P55" t="n">
         <v>0</v>
@@ -3927,10 +3927,10 @@
         <v>2</v>
       </c>
       <c r="S55" t="n">
-        <v>432</v>
+        <v>336</v>
       </c>
       <c r="T55" t="n">
-        <v>425</v>
+        <v>542</v>
       </c>
     </row>
     <row r="56">
@@ -3978,7 +3978,7 @@
         <v>1</v>
       </c>
       <c r="O56" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="P56" t="n">
         <v>0</v>
@@ -3987,10 +3987,10 @@
         <v>2</v>
       </c>
       <c r="S56" t="n">
-        <v>470</v>
+        <v>382</v>
       </c>
       <c r="T56" t="n">
-        <v>358</v>
+        <v>398</v>
       </c>
     </row>
     <row r="57">
@@ -4038,7 +4038,7 @@
         <v>0</v>
       </c>
       <c r="O57" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="P57" t="n">
         <v>0</v>
@@ -4047,10 +4047,10 @@
         <v>1</v>
       </c>
       <c r="S57" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>320</v>
+        <v>431</v>
       </c>
     </row>
     <row r="58">
@@ -4080,7 +4080,7 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" s="10" t="n"/>
       <c r="H58" t="n">
-        <v>28.5</v>
+        <v>28</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
@@ -4092,7 +4092,7 @@
         <v>0</v>
       </c>
       <c r="L58" t="n">
-        <v>28.5</v>
+        <v>28</v>
       </c>
       <c r="N58" t="n">
         <v>0</v>
@@ -4107,10 +4107,10 @@
         <v>1</v>
       </c>
       <c r="S58" t="n">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="T58" t="n">
-        <v>444</v>
+        <v>539</v>
       </c>
     </row>
     <row r="59">
@@ -4158,7 +4158,7 @@
         <v>0</v>
       </c>
       <c r="O59" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="P59" t="n">
         <v>0</v>
@@ -4167,10 +4167,10 @@
         <v>1</v>
       </c>
       <c r="S59" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>471</v>
+        <v>621</v>
       </c>
     </row>
     <row r="60">
@@ -4218,7 +4218,7 @@
         <v>1</v>
       </c>
       <c r="O60" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="P60" t="n">
         <v>0</v>
@@ -4227,10 +4227,10 @@
         <v>2</v>
       </c>
       <c r="S60" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="T60" t="n">
-        <v>435</v>
+        <v>512</v>
       </c>
     </row>
     <row r="61">
@@ -4278,7 +4278,7 @@
         <v>1</v>
       </c>
       <c r="O61" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="P61" t="n">
         <v>0</v>
@@ -4287,10 +4287,10 @@
         <v>1</v>
       </c>
       <c r="S61" t="n">
-        <v>416</v>
+        <v>329</v>
       </c>
       <c r="T61" t="n">
-        <v>320</v>
+        <v>398</v>
       </c>
     </row>
     <row r="62">
@@ -4320,7 +4320,7 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" s="10" t="n"/>
       <c r="H62" t="n">
-        <v>30</v>
+        <v>29.5</v>
       </c>
       <c r="I62" t="n">
         <v>0</v>
@@ -4332,13 +4332,13 @@
         <v>0</v>
       </c>
       <c r="L62" t="n">
-        <v>30</v>
+        <v>29.5</v>
       </c>
       <c r="N62" t="n">
         <v>1</v>
       </c>
       <c r="O62" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="P62" t="n">
         <v>0</v>
@@ -4347,10 +4347,10 @@
         <v>1</v>
       </c>
       <c r="S62" t="n">
-        <v>203</v>
+        <v>158</v>
       </c>
       <c r="T62" t="n">
-        <v>444</v>
+        <v>520</v>
       </c>
     </row>
     <row r="63">
@@ -4398,7 +4398,7 @@
         <v>4</v>
       </c>
       <c r="O63" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="P63" t="n">
         <v>0</v>
@@ -4407,10 +4407,10 @@
         <v>1</v>
       </c>
       <c r="S63" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>320</v>
+        <v>436</v>
       </c>
     </row>
     <row r="64">
@@ -4458,7 +4458,7 @@
         <v>2</v>
       </c>
       <c r="O64" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="P64" t="n">
         <v>0</v>
@@ -4467,10 +4467,10 @@
         <v>2</v>
       </c>
       <c r="S64" t="n">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="T64" t="n">
-        <v>140</v>
+        <v>217</v>
       </c>
     </row>
     <row r="65">
@@ -4527,10 +4527,10 @@
         <v>1</v>
       </c>
       <c r="S65" t="n">
-        <v>347</v>
+        <v>327</v>
       </c>
       <c r="T65" t="n">
-        <v>337</v>
+        <v>449</v>
       </c>
     </row>
     <row r="66">
@@ -4560,7 +4560,7 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" s="10" t="n"/>
       <c r="H66" t="n">
-        <v>25.5</v>
+        <v>24.5</v>
       </c>
       <c r="I66" t="n">
         <v>0</v>
@@ -4572,7 +4572,7 @@
         <v>0</v>
       </c>
       <c r="L66" t="n">
-        <v>25.5</v>
+        <v>24.5</v>
       </c>
       <c r="N66" t="n">
         <v>0</v>
@@ -4590,7 +4590,7 @@
         <v>0</v>
       </c>
       <c r="T66" t="n">
-        <v>147</v>
+        <v>256</v>
       </c>
     </row>
     <row r="67">
@@ -4650,7 +4650,7 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>452</v>
+        <v>529</v>
       </c>
     </row>
     <row r="68">
@@ -4698,7 +4698,7 @@
         <v>1</v>
       </c>
       <c r="O68" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="P68" t="n">
         <v>0</v>
@@ -4707,10 +4707,10 @@
         <v>1</v>
       </c>
       <c r="S68" t="n">
-        <v>254</v>
+        <v>159</v>
       </c>
       <c r="T68" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
     </row>
     <row r="69">
@@ -4740,7 +4740,7 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" s="10" t="n"/>
       <c r="H69" t="n">
-        <v>20</v>
+        <v>19.5</v>
       </c>
       <c r="I69" t="n">
         <v>0</v>
@@ -4752,13 +4752,13 @@
         <v>0</v>
       </c>
       <c r="L69" t="n">
-        <v>20</v>
+        <v>19.5</v>
       </c>
       <c r="N69" t="n">
         <v>6</v>
       </c>
       <c r="O69" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="P69" t="n">
         <v>0</v>
@@ -4767,10 +4767,10 @@
         <v>2</v>
       </c>
       <c r="S69" t="n">
-        <v>177</v>
+        <v>152</v>
       </c>
       <c r="T69" t="n">
-        <v>147</v>
+        <v>223</v>
       </c>
     </row>
     <row r="70">
@@ -4827,10 +4827,10 @@
         <v>3</v>
       </c>
       <c r="S70" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="T70" t="n">
-        <v>282</v>
+        <v>399</v>
       </c>
     </row>
     <row r="71">
@@ -4878,7 +4878,7 @@
         <v>0</v>
       </c>
       <c r="O71" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="P71" t="n">
         <v>0</v>
@@ -4887,10 +4887,10 @@
         <v>1</v>
       </c>
       <c r="S71" t="n">
-        <v>783</v>
+        <v>712</v>
       </c>
       <c r="T71" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="72">
@@ -4938,7 +4938,7 @@
         <v>0</v>
       </c>
       <c r="O72" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="P72" t="n">
         <v>0</v>
@@ -4947,10 +4947,10 @@
         <v>1</v>
       </c>
       <c r="S72" t="n">
-        <v>174</v>
+        <v>85</v>
       </c>
       <c r="T72" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="73">
@@ -4998,7 +4998,7 @@
         <v>1</v>
       </c>
       <c r="O73" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="P73" t="n">
         <v>0</v>
@@ -5007,10 +5007,10 @@
         <v>1</v>
       </c>
       <c r="S73" t="n">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="T73" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="74">
@@ -5058,7 +5058,7 @@
         <v>0</v>
       </c>
       <c r="O74" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="P74" t="n">
         <v>0</v>
@@ -5067,10 +5067,10 @@
         <v>1</v>
       </c>
       <c r="S74" t="n">
+        <v>13</v>
+      </c>
+      <c r="T74" t="n">
         <v>38</v>
-      </c>
-      <c r="T74" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -5118,7 +5118,7 @@
         <v>0</v>
       </c>
       <c r="O75" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="P75" t="n">
         <v>0</v>
@@ -5127,10 +5127,10 @@
         <v>1</v>
       </c>
       <c r="S75" t="n">
-        <v>177</v>
+        <v>85</v>
       </c>
       <c r="T75" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="76">
@@ -5178,7 +5178,7 @@
         <v>0</v>
       </c>
       <c r="O76" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="P76" t="n">
         <v>0</v>
@@ -5187,10 +5187,10 @@
         <v>1</v>
       </c>
       <c r="S76" t="n">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="T76" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="77">
@@ -5238,7 +5238,7 @@
         <v>0</v>
       </c>
       <c r="O77" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="P77" t="n">
         <v>0</v>
@@ -5247,10 +5247,10 @@
         <v>1</v>
       </c>
       <c r="S77" t="n">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="T77" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="78">
@@ -5298,7 +5298,7 @@
         <v>0</v>
       </c>
       <c r="O78" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="P78" t="n">
         <v>0</v>
@@ -5307,10 +5307,10 @@
         <v>1</v>
       </c>
       <c r="S78" t="n">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="T78" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="79">
@@ -5358,7 +5358,7 @@
         <v>0</v>
       </c>
       <c r="O79" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="P79" t="n">
         <v>0</v>
@@ -5367,10 +5367,10 @@
         <v>1</v>
       </c>
       <c r="S79" t="n">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="T79" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="80">
@@ -5418,7 +5418,7 @@
         <v>0</v>
       </c>
       <c r="O80" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="P80" t="n">
         <v>0</v>
@@ -5427,10 +5427,10 @@
         <v>1</v>
       </c>
       <c r="S80" t="n">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="T80" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="81">
@@ -5478,7 +5478,7 @@
         <v>1</v>
       </c>
       <c r="O81" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="P81" t="n">
         <v>0</v>
@@ -5487,7 +5487,7 @@
         <v>1</v>
       </c>
       <c r="S81" t="n">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="T81" t="n">
         <v>0</v>
@@ -5538,7 +5538,7 @@
         <v>0</v>
       </c>
       <c r="O82" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="P82" t="n">
         <v>0</v>
@@ -5547,10 +5547,10 @@
         <v>1</v>
       </c>
       <c r="S82" t="n">
-        <v>98</v>
+        <v>15</v>
       </c>
       <c r="T82" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="83">
@@ -5598,7 +5598,7 @@
         <v>0</v>
       </c>
       <c r="O83" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="P83" t="n">
         <v>0</v>
@@ -5607,10 +5607,10 @@
         <v>1</v>
       </c>
       <c r="S83" t="n">
-        <v>87</v>
+        <v>14</v>
       </c>
       <c r="T83" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="84">
@@ -5658,7 +5658,7 @@
         <v>0</v>
       </c>
       <c r="O84" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="P84" t="n">
         <v>0</v>
@@ -5667,10 +5667,10 @@
         <v>1</v>
       </c>
       <c r="S84" t="n">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="T84" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="85">
@@ -5718,7 +5718,7 @@
         <v>0</v>
       </c>
       <c r="O85" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="P85" t="n">
         <v>0</v>
@@ -5727,10 +5727,10 @@
         <v>1</v>
       </c>
       <c r="S85" t="n">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="T85" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="86">
@@ -5778,7 +5778,7 @@
         <v>1</v>
       </c>
       <c r="O86" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="P86" t="n">
         <v>0</v>
@@ -5787,10 +5787,10 @@
         <v>1</v>
       </c>
       <c r="S86" t="n">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="T86" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="87">
@@ -5838,7 +5838,7 @@
         <v>0</v>
       </c>
       <c r="O87" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="P87" t="n">
         <v>0</v>
@@ -5847,10 +5847,10 @@
         <v>1</v>
       </c>
       <c r="S87" t="n">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="T87" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="88">
@@ -5898,7 +5898,7 @@
         <v>0</v>
       </c>
       <c r="O88" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="P88" t="n">
         <v>0</v>
@@ -5907,10 +5907,10 @@
         <v>1</v>
       </c>
       <c r="S88" t="n">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="T88" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="89">
@@ -5958,7 +5958,7 @@
         <v>0</v>
       </c>
       <c r="O89" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="P89" t="n">
         <v>0</v>
@@ -5967,10 +5967,10 @@
         <v>1</v>
       </c>
       <c r="S89" t="n">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="T89" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="90">
@@ -6092,7 +6092,7 @@
         <v>0</v>
       </c>
       <c r="T91" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="92">
@@ -6140,7 +6140,7 @@
         <v>2</v>
       </c>
       <c r="O92" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="P92" t="n">
         <v>0</v>
@@ -6149,10 +6149,10 @@
         <v>1</v>
       </c>
       <c r="S92" t="n">
-        <v>358</v>
+        <v>329</v>
       </c>
       <c r="T92" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="93">
@@ -6200,7 +6200,7 @@
         <v>0</v>
       </c>
       <c r="O93" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="P93" t="n">
         <v>0</v>
@@ -6209,10 +6209,10 @@
         <v>1</v>
       </c>
       <c r="S93" t="n">
-        <v>65</v>
+        <v>1</v>
       </c>
       <c r="T93" t="n">
-        <v>318</v>
+        <v>396</v>
       </c>
     </row>
     <row r="94">
@@ -6260,7 +6260,7 @@
         <v>3</v>
       </c>
       <c r="O94" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="P94" t="n">
         <v>0</v>
@@ -6269,10 +6269,10 @@
         <v>1</v>
       </c>
       <c r="S94" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="T94" t="n">
-        <v>0</v>
+        <v>103</v>
       </c>
     </row>
     <row r="95">
@@ -6302,7 +6302,7 @@
       <c r="F95" t="inlineStr"/>
       <c r="G95" s="10" t="n"/>
       <c r="H95" t="n">
-        <v>21.5</v>
+        <v>20.5</v>
       </c>
       <c r="I95" t="n">
         <v>0</v>
@@ -6314,13 +6314,13 @@
         <v>0</v>
       </c>
       <c r="L95" t="n">
-        <v>21.5</v>
+        <v>20.5</v>
       </c>
       <c r="N95" t="n">
         <v>2</v>
       </c>
       <c r="O95" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="P95" t="n">
         <v>0</v>
@@ -6329,10 +6329,10 @@
         <v>2</v>
       </c>
       <c r="S95" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T95" t="n">
-        <v>146</v>
+        <v>260</v>
       </c>
     </row>
     <row r="96">
@@ -6380,7 +6380,7 @@
         <v>1</v>
       </c>
       <c r="O96" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="P96" t="n">
         <v>0</v>
@@ -6389,10 +6389,10 @@
         <v>1</v>
       </c>
       <c r="S96" t="n">
-        <v>97</v>
+        <v>12</v>
       </c>
       <c r="T96" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="97">
@@ -6440,7 +6440,7 @@
         <v>1</v>
       </c>
       <c r="O97" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="P97" t="n">
         <v>0</v>
@@ -6449,10 +6449,10 @@
         <v>1</v>
       </c>
       <c r="S97" t="n">
-        <v>122</v>
+        <v>20</v>
       </c>
       <c r="T97" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="98">
@@ -6482,7 +6482,7 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" s="10" t="n"/>
       <c r="H98" t="n">
-        <v>18</v>
+        <v>17.5</v>
       </c>
       <c r="I98" t="n">
         <v>0</v>
@@ -6494,7 +6494,7 @@
         <v>0</v>
       </c>
       <c r="L98" t="n">
-        <v>18</v>
+        <v>17.5</v>
       </c>
       <c r="N98" t="n">
         <v>2</v>
@@ -6512,7 +6512,7 @@
         <v>0</v>
       </c>
       <c r="T98" t="n">
-        <v>629</v>
+        <v>706</v>
       </c>
     </row>
     <row r="99">
@@ -6684,7 +6684,7 @@
         <v>1</v>
       </c>
       <c r="O101" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="P101" t="n">
         <v>0</v>
@@ -6693,10 +6693,10 @@
         <v>1</v>
       </c>
       <c r="S101" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="T101" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="102">
@@ -6744,7 +6744,7 @@
         <v>0</v>
       </c>
       <c r="O102" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="P102" t="n">
         <v>0</v>
@@ -6753,10 +6753,10 @@
         <v>1</v>
       </c>
       <c r="S102" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="103">
@@ -6816,7 +6816,7 @@
         <v>0</v>
       </c>
       <c r="T103" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="104">
@@ -6864,7 +6864,7 @@
         <v>0</v>
       </c>
       <c r="O104" t="n">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="P104" t="n">
         <v>0</v>
@@ -6873,10 +6873,10 @@
         <v>1</v>
       </c>
       <c r="S104" t="n">
-        <v>198</v>
+        <v>160</v>
       </c>
       <c r="T104" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="105">
@@ -6924,7 +6924,7 @@
         <v>3</v>
       </c>
       <c r="O105" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="P105" t="n">
         <v>0</v>
@@ -6933,10 +6933,10 @@
         <v>2</v>
       </c>
       <c r="S105" t="n">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="T105" t="n">
-        <v>318</v>
+        <v>396</v>
       </c>
     </row>
     <row r="106">
@@ -6984,7 +6984,7 @@
         <v>2</v>
       </c>
       <c r="O106" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="P106" t="n">
         <v>0</v>
@@ -6993,10 +6993,10 @@
         <v>1</v>
       </c>
       <c r="S106" t="n">
-        <v>154</v>
+        <v>51</v>
       </c>
       <c r="T106" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="107">
@@ -7026,7 +7026,7 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" s="10" t="n"/>
       <c r="H107" t="n">
-        <v>25</v>
+        <v>24.5</v>
       </c>
       <c r="I107" t="n">
         <v>0</v>
@@ -7038,7 +7038,7 @@
         <v>0</v>
       </c>
       <c r="L107" t="n">
-        <v>25</v>
+        <v>24.5</v>
       </c>
       <c r="N107" t="n">
         <v>2</v>
@@ -7053,10 +7053,10 @@
         <v>2</v>
       </c>
       <c r="S107" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="T107" t="n">
-        <v>470</v>
+        <v>550</v>
       </c>
     </row>
     <row r="108">
@@ -7113,10 +7113,10 @@
         <v>1</v>
       </c>
       <c r="S108" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="T108" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="109">
@@ -7164,7 +7164,7 @@
         <v>1</v>
       </c>
       <c r="O109" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="P109" t="n">
         <v>0</v>
@@ -7173,10 +7173,10 @@
         <v>1</v>
       </c>
       <c r="S109" t="n">
-        <v>263</v>
+        <v>159</v>
       </c>
       <c r="T109" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="110">
@@ -7224,7 +7224,7 @@
         <v>2</v>
       </c>
       <c r="O110" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="P110" t="n">
         <v>0</v>
@@ -7233,10 +7233,10 @@
         <v>1</v>
       </c>
       <c r="S110" t="n">
-        <v>178</v>
+        <v>151</v>
       </c>
       <c r="T110" t="n">
-        <v>320</v>
+        <v>396</v>
       </c>
     </row>
     <row r="111">
@@ -7284,7 +7284,7 @@
         <v>0</v>
       </c>
       <c r="O111" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="P111" t="n">
         <v>0</v>
@@ -7293,10 +7293,10 @@
         <v>1</v>
       </c>
       <c r="S111" t="n">
-        <v>435</v>
+        <v>388</v>
       </c>
       <c r="T111" t="n">
-        <v>0</v>
+        <v>69</v>
       </c>
     </row>
     <row r="112">
@@ -7344,7 +7344,7 @@
         <v>1</v>
       </c>
       <c r="O112" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="P112" t="n">
         <v>0</v>
@@ -7353,10 +7353,10 @@
         <v>1</v>
       </c>
       <c r="S112" t="n">
-        <v>207</v>
+        <v>172</v>
       </c>
       <c r="T112" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="113">
@@ -7404,7 +7404,7 @@
         <v>0</v>
       </c>
       <c r="O113" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="P113" t="n">
         <v>0</v>
@@ -7413,10 +7413,10 @@
         <v>1</v>
       </c>
       <c r="S113" t="n">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="T113" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="114">
@@ -7464,7 +7464,7 @@
         <v>0</v>
       </c>
       <c r="O114" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="P114" t="n">
         <v>0</v>
@@ -7473,10 +7473,10 @@
         <v>1</v>
       </c>
       <c r="S114" t="n">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="T114" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="115">
@@ -7524,7 +7524,7 @@
         <v>0</v>
       </c>
       <c r="O115" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="P115" t="n">
         <v>0</v>
@@ -7533,10 +7533,10 @@
         <v>1</v>
       </c>
       <c r="S115" t="n">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="T115" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="116">
@@ -7584,7 +7584,7 @@
         <v>0</v>
       </c>
       <c r="O116" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="P116" t="n">
         <v>0</v>
@@ -7593,10 +7593,10 @@
         <v>1</v>
       </c>
       <c r="S116" t="n">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="T116" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="117">
@@ -7644,7 +7644,7 @@
         <v>0</v>
       </c>
       <c r="O117" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="P117" t="n">
         <v>0</v>
@@ -7653,10 +7653,10 @@
         <v>1</v>
       </c>
       <c r="S117" t="n">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="T117" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="118">
@@ -7704,7 +7704,7 @@
         <v>0</v>
       </c>
       <c r="O118" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="P118" t="n">
         <v>0</v>
@@ -7713,10 +7713,10 @@
         <v>1</v>
       </c>
       <c r="S118" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="T118" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="119">
@@ -7764,7 +7764,7 @@
         <v>3</v>
       </c>
       <c r="O119" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="P119" t="n">
         <v>0</v>
@@ -7773,10 +7773,10 @@
         <v>1</v>
       </c>
       <c r="S119" t="n">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="T119" t="n">
-        <v>320</v>
+        <v>398</v>
       </c>
     </row>
     <row r="120">
@@ -7824,7 +7824,7 @@
         <v>0</v>
       </c>
       <c r="O120" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="P120" t="n">
         <v>0</v>
@@ -7833,10 +7833,10 @@
         <v>1</v>
       </c>
       <c r="S120" t="n">
-        <v>96</v>
+        <v>14</v>
       </c>
       <c r="T120" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="121">
@@ -7884,7 +7884,7 @@
         <v>0</v>
       </c>
       <c r="O121" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="P121" t="n">
         <v>0</v>
@@ -7893,10 +7893,10 @@
         <v>1</v>
       </c>
       <c r="S121" t="n">
-        <v>72</v>
+        <v>15</v>
       </c>
       <c r="T121" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="122">
@@ -7944,7 +7944,7 @@
         <v>0</v>
       </c>
       <c r="O122" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="P122" t="n">
         <v>0</v>
@@ -7953,10 +7953,10 @@
         <v>1</v>
       </c>
       <c r="S122" t="n">
-        <v>90</v>
+        <v>14</v>
       </c>
       <c r="T122" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="123">
@@ -8004,7 +8004,7 @@
         <v>0</v>
       </c>
       <c r="O123" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="P123" t="n">
         <v>0</v>
@@ -8013,10 +8013,10 @@
         <v>1</v>
       </c>
       <c r="S123" t="n">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="T123" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="124">
@@ -8064,7 +8064,7 @@
         <v>0</v>
       </c>
       <c r="O124" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="P124" t="n">
         <v>0</v>
@@ -8073,10 +8073,10 @@
         <v>1</v>
       </c>
       <c r="S124" t="n">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="T124" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="125">
@@ -8124,7 +8124,7 @@
         <v>0</v>
       </c>
       <c r="O125" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="P125" t="n">
         <v>0</v>
@@ -8133,10 +8133,10 @@
         <v>1</v>
       </c>
       <c r="S125" t="n">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="T125" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="126">
@@ -8184,7 +8184,7 @@
         <v>0</v>
       </c>
       <c r="O126" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="P126" t="n">
         <v>0</v>
@@ -8193,10 +8193,10 @@
         <v>1</v>
       </c>
       <c r="S126" t="n">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="T126" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="127">
@@ -8244,7 +8244,7 @@
         <v>1</v>
       </c>
       <c r="O127" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="P127" t="n">
         <v>0</v>
@@ -8253,10 +8253,10 @@
         <v>1</v>
       </c>
       <c r="S127" t="n">
-        <v>77</v>
+        <v>13</v>
       </c>
       <c r="T127" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="128">
@@ -8304,7 +8304,7 @@
         <v>0</v>
       </c>
       <c r="O128" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="P128" t="n">
         <v>0</v>
@@ -8313,10 +8313,10 @@
         <v>1</v>
       </c>
       <c r="S128" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="T128" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="129">
@@ -8364,7 +8364,7 @@
         <v>0</v>
       </c>
       <c r="O129" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="P129" t="n">
         <v>0</v>
@@ -8373,10 +8373,10 @@
         <v>1</v>
       </c>
       <c r="S129" t="n">
-        <v>90</v>
+        <v>14</v>
       </c>
       <c r="T129" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="130">
@@ -8486,7 +8486,7 @@
         <v>1</v>
       </c>
       <c r="O131" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="P131" t="n">
         <v>0</v>
@@ -8495,7 +8495,7 @@
         <v>1</v>
       </c>
       <c r="S131" t="n">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="T131" t="n">
         <v>0</v>
@@ -8546,7 +8546,7 @@
         <v>1</v>
       </c>
       <c r="O132" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="P132" t="n">
         <v>0</v>
@@ -8555,7 +8555,7 @@
         <v>0</v>
       </c>
       <c r="S132" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="T132" t="n">
         <v>0</v>
@@ -8606,7 +8606,7 @@
         <v>1</v>
       </c>
       <c r="O133" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="P133" t="n">
         <v>0</v>
@@ -8615,7 +8615,7 @@
         <v>0</v>
       </c>
       <c r="S133" t="n">
-        <v>71</v>
+        <v>14</v>
       </c>
       <c r="T133" t="n">
         <v>0</v>
@@ -8666,19 +8666,19 @@
         <v>1</v>
       </c>
       <c r="O134" t="n">
+        <v>30</v>
+      </c>
+      <c r="P134" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q134" t="n">
+        <v>1</v>
+      </c>
+      <c r="S134" t="n">
         <v>3</v>
       </c>
-      <c r="P134" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q134" t="n">
-        <v>1</v>
-      </c>
-      <c r="S134" t="n">
-        <v>80</v>
-      </c>
       <c r="T134" t="n">
-        <v>39</v>
+        <v>79</v>
       </c>
     </row>
     <row r="135">
@@ -8726,7 +8726,7 @@
         <v>1</v>
       </c>
       <c r="O135" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="P135" t="n">
         <v>0</v>
@@ -8735,10 +8735,10 @@
         <v>1</v>
       </c>
       <c r="S135" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="T135" t="n">
-        <v>347</v>
+        <v>387</v>
       </c>
     </row>
     <row r="136">
@@ -8786,7 +8786,7 @@
         <v>1</v>
       </c>
       <c r="O136" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="P136" t="n">
         <v>0</v>
@@ -8795,10 +8795,10 @@
         <v>1</v>
       </c>
       <c r="S136" t="n">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="T136" t="n">
-        <v>347</v>
+        <v>387</v>
       </c>
     </row>
     <row r="137">
@@ -8906,7 +8906,7 @@
         <v>1</v>
       </c>
       <c r="O138" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="P138" t="n">
         <v>0</v>
@@ -8915,10 +8915,10 @@
         <v>1</v>
       </c>
       <c r="S138" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="T138" t="n">
-        <v>347</v>
+        <v>387</v>
       </c>
     </row>
     <row r="139">
@@ -9266,7 +9266,7 @@
         <v>0</v>
       </c>
       <c r="O144" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="P144" t="n">
         <v>0</v>
@@ -9275,10 +9275,10 @@
         <v>1</v>
       </c>
       <c r="S144" t="n">
-        <v>137</v>
+        <v>32</v>
       </c>
       <c r="T144" t="n">
-        <v>228</v>
+        <v>268</v>
       </c>
     </row>
     <row r="145">
@@ -9335,10 +9335,10 @@
         <v>2</v>
       </c>
       <c r="S145" t="n">
-        <v>259</v>
+        <v>129</v>
       </c>
       <c r="T145" t="n">
-        <v>322</v>
+        <v>505</v>
       </c>
     </row>
     <row r="146">
@@ -9506,7 +9506,7 @@
         <v>0</v>
       </c>
       <c r="O148" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="P148" t="n">
         <v>0</v>
@@ -9746,7 +9746,7 @@
         <v>3</v>
       </c>
       <c r="O152" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P152" t="n">
         <v>0</v>
@@ -9806,7 +9806,7 @@
         <v>1</v>
       </c>
       <c r="O153" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="P153" t="n">
         <v>0</v>
@@ -9866,7 +9866,7 @@
         <v>1</v>
       </c>
       <c r="O154" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="P154" t="n">
         <v>0</v>
@@ -9986,7 +9986,7 @@
         <v>0</v>
       </c>
       <c r="O156" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="P156" t="n">
         <v>0</v>
@@ -10106,7 +10106,7 @@
         <v>0</v>
       </c>
       <c r="O158" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="P158" t="n">
         <v>0</v>
@@ -10115,10 +10115,10 @@
         <v>1</v>
       </c>
       <c r="S158" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="T158" t="n">
-        <v>434</v>
+        <v>523</v>
       </c>
     </row>
     <row r="159">
@@ -10408,7 +10408,7 @@
         <v>2</v>
       </c>
       <c r="O163" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="P163" t="n">
         <v>0</v>

</xml_diff>